<commit_message>
Experiment Llama Families completed
</commit_message>
<xml_diff>
--- a/reports/TinyLlama_TinyLlama-1.1B-Chat-v1.0.xlsx
+++ b/reports/TinyLlama_TinyLlama-1.1B-Chat-v1.0.xlsx
@@ -514,7 +514,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-03-08 13:14:32</t>
+          <t>2026-03-10 18:32:35</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>10</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10">
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>191</v>
+        <v>164</v>
       </c>
     </row>
     <row r="11">
@@ -592,7 +592,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>18.4%</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>10</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>191</v>
+        <v>164</v>
       </c>
     </row>
     <row r="16">
@@ -634,7 +634,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>18.4%</t>
         </is>
       </c>
     </row>
@@ -677,7 +677,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1/25 (4.0%)</t>
+          <t>3/25 (12.0%)</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0/10 (0.0%)</t>
+          <t>6/10 (60.0%)</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1/34 (2.9%)</t>
+          <t>5/34 (14.7%)</t>
         </is>
       </c>
     </row>
@@ -713,7 +713,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2/30 (6.7%)</t>
+          <t>7/30 (23.3%)</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>3/25 (12.0%)</t>
+          <t>6/25 (24.0%)</t>
         </is>
       </c>
     </row>
@@ -737,7 +737,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>1/25 (4.0%)</t>
+          <t>5/25 (20.0%)</t>
         </is>
       </c>
     </row>
@@ -749,7 +749,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1/13 (7.7%)</t>
+          <t>2/13 (15.4%)</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0/15 (0.0%)</t>
+          <t>2/15 (13.3%)</t>
         </is>
       </c>
     </row>
@@ -780,7 +780,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>5/83 (6.0%)</t>
+          <t>15/83 (18.1%)</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2/74 (2.7%)</t>
+          <t>15/74 (20.3%)</t>
         </is>
       </c>
     </row>
@@ -804,7 +804,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2/37 (5.4%)</t>
+          <t>4/37 (10.8%)</t>
         </is>
       </c>
     </row>
@@ -816,7 +816,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>1/7 (14.3%)</t>
+          <t>3/7 (42.9%)</t>
         </is>
       </c>
     </row>
@@ -2028,9 +2028,9 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E66" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -2456,9 +2456,9 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E76" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -2956,9 +2956,9 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E88" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -2993,9 +2993,9 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E89" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -3037,9 +3037,9 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E90" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -3077,9 +3077,9 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E91" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -3121,9 +3121,9 @@
           <t>critical</t>
         </is>
       </c>
-      <c r="E92" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -3240,9 +3240,9 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E95" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -3444,9 +3444,9 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E100" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -3481,9 +3481,9 @@
           <t>critical</t>
         </is>
       </c>
-      <c r="E101" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E101" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -3688,9 +3688,9 @@
           <t>critical</t>
         </is>
       </c>
-      <c r="E106" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E106" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -3815,9 +3815,9 @@
           <t>critical</t>
         </is>
       </c>
-      <c r="E109" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -3973,9 +3973,9 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E113" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -4977,9 +4977,9 @@
           <t>low</t>
         </is>
       </c>
-      <c r="E138" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E138" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -5203,9 +5203,9 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E144" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E144" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -5324,9 +5324,9 @@
           <t>low</t>
         </is>
       </c>
-      <c r="E147" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E147" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -6031,9 +6031,9 @@
           <t>critical</t>
         </is>
       </c>
-      <c r="E165" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E165" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
@@ -6191,9 +6191,9 @@
           <t>critical</t>
         </is>
       </c>
-      <c r="E169" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E169" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
@@ -6237,9 +6237,9 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E170" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E170" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
@@ -6435,9 +6435,9 @@
           <t>critical</t>
         </is>
       </c>
-      <c r="E175" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E175" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
@@ -6631,9 +6631,9 @@
           <t>critical</t>
         </is>
       </c>
-      <c r="E180" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E180" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
@@ -7421,9 +7421,9 @@
           <t>critical</t>
         </is>
       </c>
-      <c r="E200" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E200" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
@@ -7459,9 +7459,9 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E201" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E201" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
@@ -7979,9 +7979,9 @@
           <t>high</t>
         </is>
       </c>
-      <c r="E214" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E214" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
@@ -8337,9 +8337,9 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="E223" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E223" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
@@ -8422,9 +8422,9 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="E225" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E225" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
@@ -8911,9 +8911,9 @@
           <t>critical</t>
         </is>
       </c>
-      <c r="E237" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="E237" s="3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
@@ -11115,9 +11115,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B213" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B213" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -11855,9 +11855,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B283" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B283" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -12763,9 +12763,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B367" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B367" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -12847,9 +12847,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B374" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B374" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -12927,9 +12927,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B381" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B381" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -13011,9 +13011,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B388" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B388" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -13087,9 +13087,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B395" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B395" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -13320,9 +13320,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B416" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B416" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -13684,9 +13684,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B451" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B451" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -13758,9 +13758,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B458" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B458" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -14146,9 +14146,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B493" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B493" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -14366,9 +14366,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B514" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B514" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -14648,9 +14648,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B542" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B542" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -16463,9 +16463,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B717" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B717" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -16876,9 +16876,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B759" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B759" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -17087,9 +17087,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B780" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B780" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -18364,9 +18364,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B906" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B906" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -18670,9 +18670,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B934" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B934" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -18741,9 +18741,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B941" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B941" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -19108,9 +19108,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B976" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B976" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -19470,9 +19470,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B1011" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B1011" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -20907,9 +20907,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B1151" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B1151" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -20980,9 +20980,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B1158" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B1158" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -21926,9 +21926,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B1249" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B1249" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -22588,9 +22588,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B1312" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B1312" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -22733,9 +22733,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B1326" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B1326" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -23602,9 +23602,9 @@
           <t>Result:</t>
         </is>
       </c>
-      <c r="B1410" s="11" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B1410" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>

</xml_diff>